<commit_message>
add md ali details
</commit_message>
<xml_diff>
--- a/public/jamin_record.xlsx
+++ b/public/jamin_record.xlsx
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Appinventiv\Desktop\jamin\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{045C5C0D-9EDA-4735-B41E-CB23B1B03EFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5945CA91-8F81-49A8-A0F2-986A998FB976}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="engineer Dada details" sheetId="1" r:id="rId1"/>
-    <sheet name="Md. Dada details" sheetId="2" r:id="rId2"/>
+    <sheet name="Md_Ali_details" sheetId="2" r:id="rId2"/>
     <sheet name="M.k.khan Details" sheetId="3" r:id="rId3"/>
     <sheet name="bade dada details" sheetId="4" r:id="rId4"/>
     <sheet name="master dada details" sheetId="5" r:id="rId5"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="219" uniqueCount="119">
   <si>
     <t>0.3.7</t>
   </si>
@@ -387,6 +387,15 @@
   </si>
   <si>
     <t>Wrong in the list that is  0.3.9 rest addin md. Ali</t>
+  </si>
+  <si>
+    <t>Removed and Added in M.k.khan</t>
+  </si>
+  <si>
+    <t>0.2.9</t>
+  </si>
+  <si>
+    <t>Added in Md Ali 0.2.9</t>
   </si>
 </sst>
 </file>
@@ -943,204 +952,431 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:G22"/>
   <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="2" width="12.6328125" style="3"/>
+    <col min="6" max="6" width="29.54296875" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="3">
+        <v>1047</v>
+      </c>
+      <c r="B2" s="3">
+        <v>9879</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1">
-        <f t="shared" ref="B1:B20" si="0">LEFT(A1,FIND(".",A1)-1)*400 + MID(A1,FIND(".",A1)+1,FIND(".",A1,FIND(".",A1)+1)-FIND(".",A1)-1)*20 + RIGHT(A1,LEN(A1)-FIND(".",A1,FIND(".",A1)+1))</f>
-        <v>67</v>
-      </c>
-      <c r="C1" s="1">
-        <f>SUM(B:B)</f>
-        <v>2096</v>
-      </c>
-      <c r="D1" s="1" t="str">
-        <f>INT(C1/400) &amp; "." &amp; INT(MOD(C1,400)/20) &amp; "." &amp; MOD(MOD(C1,400),20)</f>
-        <v>5.4.16</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+      <c r="D2" s="1">
+        <f>IF(C2="","",VALUE(_xlfn.TEXTBEFORE(C2,"."))*60+VALUE(_xlfn.TEXTBEFORE(_xlfn.TEXTAFTER(C2,"."),"."))*7.5+VALUE(_xlfn.TEXTAFTER(C2,".",2))*0.375)</f>
+        <v>25.125</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="F2" s="1"/>
+    </row>
+    <row r="3" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="3">
+        <v>1047</v>
+      </c>
+      <c r="B3" s="3">
+        <v>9855</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="1">
-        <f t="shared" si="0"/>
-        <v>447</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
+      <c r="D3" s="1">
+        <f t="shared" ref="D3:D22" si="0">IF(C3="","",VALUE(_xlfn.TEXTBEFORE(C3,"."))*60+VALUE(_xlfn.TEXTBEFORE(_xlfn.TEXTAFTER(C3,"."),"."))*7.5+VALUE(_xlfn.TEXTAFTER(C3,".",2))*0.375)</f>
+        <v>77.625</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="F3" s="1"/>
+    </row>
+    <row r="4" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="3">
+        <v>1047</v>
+      </c>
+      <c r="B4" s="3">
+        <v>9839</v>
+      </c>
+      <c r="C4" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B3" s="1">
-        <f t="shared" si="0"/>
-        <v>119</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
+      <c r="D4" s="1">
+        <f t="shared" si="0"/>
+        <v>44.625</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="3">
+        <v>1450</v>
+      </c>
+      <c r="B5" s="3">
+        <v>7027</v>
+      </c>
+      <c r="C5" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="1">
-        <f t="shared" si="0"/>
-        <v>70</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
+      <c r="D5" s="1">
+        <f t="shared" si="0"/>
+        <v>26.25</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="3">
+        <v>1450</v>
+      </c>
+      <c r="B6" s="3">
+        <v>9760</v>
+      </c>
+      <c r="C6" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="1">
-        <f t="shared" si="0"/>
-        <v>67</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
+      <c r="D6" s="1">
+        <f t="shared" si="0"/>
+        <v>25.125</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="3">
+        <v>1451</v>
+      </c>
+      <c r="B7" s="3">
+        <v>9629</v>
+      </c>
+      <c r="C7" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B6" s="1">
-        <f t="shared" si="0"/>
-        <v>19</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
+      <c r="D7" s="1">
+        <f t="shared" si="0"/>
+        <v>7.125</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="3">
+        <v>1451</v>
+      </c>
+      <c r="B8" s="3">
+        <v>9486</v>
+      </c>
+      <c r="C8" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B7" s="1">
-        <f t="shared" si="0"/>
-        <v>100</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="B8" s="1">
-        <f t="shared" si="0"/>
-        <v>66</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B9" s="1">
-        <f t="shared" si="0"/>
-        <v>68</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
+      <c r="D8" s="1">
+        <f t="shared" si="0"/>
+        <v>37.5</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="3">
+        <v>1451</v>
+      </c>
+      <c r="B9" s="3">
+        <v>9467</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="D9" s="1">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="E9" t="s">
+        <v>81</v>
+      </c>
+      <c r="F9" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="3">
+        <v>1451</v>
+      </c>
+      <c r="B10" s="3">
+        <v>9466</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="D10" s="1">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="E10" t="s">
+        <v>81</v>
+      </c>
+      <c r="F10" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="3">
+        <v>1452</v>
+      </c>
+      <c r="B11" s="3">
+        <v>9835</v>
+      </c>
+      <c r="C11" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="B10" s="1">
-        <f t="shared" si="0"/>
-        <v>52</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="s">
+      <c r="D11" s="1">
+        <f t="shared" si="0"/>
+        <v>19.5</v>
+      </c>
+      <c r="E11" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="3">
+        <v>1452</v>
+      </c>
+      <c r="B12" s="3">
+        <v>9805</v>
+      </c>
+      <c r="C12" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="B11" s="1">
-        <f t="shared" si="0"/>
-        <v>27</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="1" t="s">
+      <c r="D12" s="1">
+        <f t="shared" si="0"/>
+        <v>10.125</v>
+      </c>
+      <c r="E12" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="3">
+        <v>1452</v>
+      </c>
+      <c r="B13" s="3">
+        <v>9807</v>
+      </c>
+      <c r="C13" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="B12" s="1">
-        <f t="shared" si="0"/>
-        <v>47</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="1" t="s">
+      <c r="D13" s="1">
+        <f t="shared" si="0"/>
+        <v>17.625</v>
+      </c>
+      <c r="E13" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="3">
+        <v>1452</v>
+      </c>
+      <c r="B14" s="3">
+        <v>9599</v>
+      </c>
+      <c r="C14" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="B13" s="1">
-        <f t="shared" si="0"/>
-        <v>32</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="1" t="s">
+      <c r="D14" s="1">
+        <f t="shared" si="0"/>
+        <v>12</v>
+      </c>
+      <c r="E14" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="3">
+        <v>1452</v>
+      </c>
+      <c r="B15" s="3">
+        <v>9600</v>
+      </c>
+      <c r="C15" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B14" s="1">
-        <f t="shared" si="0"/>
+      <c r="D15" s="1">
+        <f t="shared" si="0"/>
+        <v>10.875</v>
+      </c>
+      <c r="E15" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="3">
+        <v>1452</v>
+      </c>
+      <c r="B16" s="3">
+        <v>9596</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D16" s="1">
+        <f t="shared" si="0"/>
+        <v>76.5</v>
+      </c>
+      <c r="E16" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="3">
+        <v>1452</v>
+      </c>
+      <c r="B17" s="3">
+        <v>9781</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D17" s="1">
+        <f t="shared" si="0"/>
+        <v>17.625</v>
+      </c>
+      <c r="E17" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="3">
+        <v>1452</v>
+      </c>
+      <c r="B18" s="3">
+        <v>9782</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D18" s="1">
+        <f t="shared" si="0"/>
+        <v>29.625</v>
+      </c>
+      <c r="E18" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="3">
+        <v>1452</v>
+      </c>
+      <c r="B19" s="3">
+        <v>9614</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="D19" s="1">
+        <f t="shared" si="0"/>
+        <v>82.5</v>
+      </c>
+      <c r="E19" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="3">
+        <v>2007</v>
+      </c>
+      <c r="B20" s="3">
+        <v>9746</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="D20" s="1">
+        <f t="shared" si="0"/>
+        <v>82.5</v>
+      </c>
+      <c r="E20" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A21" s="3">
+        <v>1173</v>
+      </c>
+      <c r="B21" s="3">
+        <v>9875</v>
+      </c>
+      <c r="C21" s="1" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="15" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="B15" s="1">
-        <f t="shared" si="0"/>
-        <v>204</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="B16" s="1">
-        <f t="shared" si="0"/>
-        <v>47</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="B17" s="1">
-        <f t="shared" si="0"/>
-        <v>79</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="B18" s="1">
-        <f t="shared" si="0"/>
-        <v>220</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="B19" s="1">
-        <f t="shared" si="0"/>
-        <v>220</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A20" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="B20" s="1">
-        <f t="shared" si="0"/>
-        <v>116</v>
+      <c r="D21" s="1">
+        <f t="shared" si="0"/>
+        <v>43.5</v>
+      </c>
+      <c r="E21" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="3">
+        <v>1452</v>
+      </c>
+      <c r="B22" s="3">
+        <v>9766</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="D22" s="1">
+        <f t="shared" si="0"/>
+        <v>18.375</v>
+      </c>
+      <c r="E22" t="s">
+        <v>81</v>
+      </c>
+      <c r="F22" t="s">
+        <v>118</v>
       </c>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E1:E1048576" xr:uid="{0A2671B1-1588-4FF0-9B05-702F684C477A}">
+      <formula1>"Correct,Disputed"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>